<commit_message>
Lecture 4: final class version (72 slides) — slide refs renumbered, 9 quick checks rebuilt as practice questions
</commit_message>
<xml_diff>
--- a/docs/sketch/kahoot/unit2_L04.xlsx
+++ b/docs/sketch/kahoot/unit2_L04.xlsx
@@ -2725,35 +2725,35 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>Which pairing correctly matches a drug with its primary mechanism?</t>
+          <t>Based on Figure 7, which bisphosphonate requires the fewest doses per year, and by what route is it given?</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Methotrexate — dihydrofolate reductase inhibition</t>
+          <t>Ibandronate, given orally</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Allopurinol — microtubule disruption</t>
+          <t>Alendronate/risedronate, given orally</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>Colchicine — xanthine oxidase inhibition</t>
+          <t>All bisphosphonates require the same number of annual doses</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
-          <t>Baclofen — calcium channel blockade in skeletal muscle</t>
+          <t>Zoledronic acid, given intravenously</t>
         </is>
       </c>
       <c r="G24" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H24" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I24" s="1" t="n"/>
@@ -2782,27 +2782,27 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>A patient on a biologic DMARD develops a fever. What is the most important immediate concern?</t>
+          <t>Which pairing correctly matches a drug with its primary mechanism?</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>Infection, given the drug’s immunosuppressive effect</t>
+          <t>Methotrexate — dihydrofolate reductase inhibition</t>
         </is>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>Osteonecrosis of the jaw</t>
+          <t>Allopurinol — microtubule disruption</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Hepatotoxicity from Phase II metabolism</t>
+          <t>Baclofen — calcium channel blockade in skeletal muscle</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>A drug allergy only</t>
+          <t>Colchicine — xanthine oxidase inhibition</t>
         </is>
       </c>
       <c r="G25" s="14" t="n">
@@ -2839,27 +2839,27 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Which statement correctly contrasts how allopurinol and probenecid lower serum uric acid?</t>
+          <t>A patient on a biologic DMARD develops a fever. What is the most important immediate concern?</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Both inhibit xanthine oxidase at different sites</t>
+          <t>Osteonecrosis of the jaw</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>Allopurinol raises excretion; probenecid cuts production</t>
+          <t>A drug allergy only</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Allopurinol blocks neutrophils; probenecid blocks URAT1</t>
+          <t>Hepatotoxicity from Phase II metabolism</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>Allopurinol cuts production; probenecid raises renal excretion</t>
+          <t>Infection, given the drug’s immunosuppressive effect</t>
         </is>
       </c>
       <c r="G26" s="14" t="n">
@@ -2901,22 +2901,22 @@
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
+          <t>It inhibits xanthine oxidase, lowering uric acid</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>It blocks URAT1, increasing uric acid excretion</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>It disrupts microtubules, reducing neutrophil migration</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
           <t>It converts uric acid to allantoin in the joint</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>It inhibits xanthine oxidase, lowering uric acid</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>It blocks phospholipase A₂ upstream of COX</t>
-        </is>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>It disrupts microtubules, reducing neutrophil migration</t>
         </is>
       </c>
       <c r="G27" s="14" t="n">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="H27" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I27" s="1" t="n"/>
@@ -2958,22 +2958,22 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
+          <t>Clarithromycin triggers HLA-B*58:01 hypersensitivity</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>CYP3A4/P-gp inhibition raises colchicine to toxic levels</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
           <t>The two together cause hemolysis in G6PD deficiency</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>Clarithromycin triggers HLA-B*58:01 hypersensitivity</t>
-        </is>
-      </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>Clarithromycin speeds colchicine clearance, so the flare returns</t>
-        </is>
-      </c>
-      <c r="F28" s="14" t="inlineStr">
-        <is>
-          <t>CYP3A4/P-gp inhibition raises colchicine to toxic levels</t>
         </is>
       </c>
       <c r="G28" s="14" t="n">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="H28" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I28" s="1" t="n"/>
@@ -3015,17 +3015,17 @@
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
+          <t>Liver enzymes, because of hepatotoxicity</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
           <t>HLA-B*58:01, because of skin reactions</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr">
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>G6PD activity, because of hemolysis risk</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>A 24-hour urine urate, to rule out stones</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="H29" s="17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I29" s="1" t="n"/>
@@ -3072,22 +3072,22 @@
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
+          <t>Allopurinol is not used at all in CKD</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>800 mg/d, the usual maximum dose</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
           <t>100 mg/d, the same as normal kidney function</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
+      <c r="F30" s="16" t="inlineStr">
         <is>
           <t>No more than 50 mg/d, titrated by 50 mg</t>
-        </is>
-      </c>
-      <c r="E30" s="16" t="inlineStr">
-        <is>
-          <t>Allopurinol is not used at all in CKD</t>
-        </is>
-      </c>
-      <c r="F30" s="16" t="inlineStr">
-        <is>
-          <t>300 mg/d from day one to reach target fast</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="H30" s="17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I30" s="1" t="n"/>
@@ -3124,27 +3124,27 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>Which skeletal muscle relaxant acts outside the CNS, directly on the muscle fiber?</t>
+          <t>A patient taking tizanidine for spasticity is prescribed ciprofloxacin for a urinary infection. What is the problem?</t>
         </is>
       </c>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>Dantrolene</t>
+          <t>Tizanidine stops ciprofloxacin being absorbed</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>Tizanidine</t>
+          <t>The pair causes serotonin syndrome</t>
         </is>
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>Cyclobenzaprine</t>
+          <t>CYP1A2 inhibition sharply raises tizanidine levels</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
-          <t>Carisoprodol</t>
+          <t>Ciprofloxacin induces CYP1A2, so spasticity returns</t>
         </is>
       </c>
       <c r="G31" s="14" t="n">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I31" s="1" t="n"/>
@@ -3181,31 +3181,31 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>A patient taking tizanidine for spasticity is prescribed ciprofloxacin for a urinary infection. What is the problem?</t>
+          <t>A 78-year-old asks for cyclobenzaprine for back spasm. Which concern is most specific to this drug in an older adult?</t>
         </is>
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
-          <t>Tizanidine stops ciprofloxacin being absorbed</t>
+          <t>Hemolysis in a patient with G6PD deficiency</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>The pair causes serotonin syndrome</t>
+          <t>Hepatotoxicity requiring routine LFT monitoring</t>
         </is>
       </c>
       <c r="E32" s="16" t="inlineStr">
         <is>
-          <t>Ciprofloxacin induces CYP1A2, so spasticity returns</t>
+          <t>Malignant hyperthermia during later anesthesia</t>
         </is>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
-          <t>CYP1A2 inhibition sharply raises tizanidine levels</t>
+          <t>Anticholinergic confusion and urinary retention</t>
         </is>
       </c>
       <c r="G32" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H32" s="17" t="inlineStr">
         <is>
@@ -3238,35 +3238,35 @@
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>A 78-year-old asks for cyclobenzaprine for back spasm. Which concern is most specific to this drug in an older adult?</t>
+          <t>Which agent is a Schedule IV controlled substance because it is metabolized to meprobamate?</t>
         </is>
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>Hemolysis in a patient with G6PD deficiency</t>
+          <t>Carisoprodol</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>Hepatotoxicity requiring routine LFT monitoring</t>
+          <t>Tizanidine</t>
         </is>
       </c>
       <c r="E33" s="16" t="inlineStr">
         <is>
-          <t>Anticholinergic confusion and urinary retention</t>
+          <t>Chlorzoxazone</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
-          <t>Malignant hyperthermia during later anesthesia</t>
+          <t>Methocarbamol</t>
         </is>
       </c>
       <c r="G33" s="14" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H33" s="17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I33" s="1" t="n"/>
@@ -3295,27 +3295,27 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>Which agent is a Schedule IV controlled substance because it is metabolized to meprobamate?</t>
+          <t>A young man with extensive burns needs emergency intubation. Why is succinylcholine avoided?</t>
         </is>
       </c>
       <c r="C34" s="16" t="inlineStr">
         <is>
-          <t>Carisoprodol</t>
+          <t>It lasts many hours in burned patients</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>Methocarbamol</t>
+          <t>Burns make it a nondepolarizing blocker</t>
         </is>
       </c>
       <c r="E34" s="16" t="inlineStr">
         <is>
-          <t>Chlorzoxazone</t>
+          <t>It is reversed too quickly by sugammadex</t>
         </is>
       </c>
       <c r="F34" s="16" t="inlineStr">
         <is>
-          <t>Tizanidine</t>
+          <t>Potassium release can cause cardiac arrest</t>
         </is>
       </c>
       <c r="G34" s="14" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="H34" s="17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I34" s="1" t="n"/>
@@ -3352,31 +3352,31 @@
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>A young man with extensive burns needs emergency intubation. Why is succinylcholine avoided?</t>
+          <t>A 66-year-old woman starts weekly alendronate. Which counseling point most reduces her risk of esophageal injury?</t>
         </is>
       </c>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>It cannot reach the burned muscle tissue</t>
+          <t>Lie down for 30 minutes after the dose</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>Burns make it a nondepolarizing blocker</t>
+          <t>Take it with coffee to speed gastric emptying</t>
         </is>
       </c>
       <c r="E35" s="16" t="inlineStr">
         <is>
-          <t>It is reversed too quickly by sugammadex</t>
+          <t>Take it with breakfast to protect the stomach</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
-          <t>Potassium release can cause cardiac arrest</t>
+          <t>Full glass of plain water, then stay upright 30 minutes</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
@@ -3409,35 +3409,35 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>A 66-year-old woman starts weekly alendronate. Which counseling point most reduces her risk of esophageal injury?</t>
+          <t>Which osteoporosis drug is an anabolic PTH analog that stimulates osteoblast bone formation?</t>
         </is>
       </c>
       <c r="C36" s="16" t="inlineStr">
         <is>
-          <t>Full glass of plain water, then stay upright 30 minutes</t>
+          <t>Raloxifene</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>Take it with coffee to speed gastric emptying</t>
+          <t>Teriparatide</t>
         </is>
       </c>
       <c r="E36" s="16" t="inlineStr">
         <is>
-          <t>Take it with breakfast to protect the stomach</t>
+          <t>Denosumab</t>
         </is>
       </c>
       <c r="F36" s="16" t="inlineStr">
         <is>
-          <t>Take it at bedtime with a calcium supplement</t>
+          <t>Calcitonin</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I36" s="1" t="n"/>
@@ -3466,35 +3466,35 @@
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>Which osteoporosis drug is an anabolic PTH analog that stimulates osteoblast bone formation?</t>
+          <t>A patient on denosumab for 4 years wants to stop it because of the injections. What should the PA advise?</t>
         </is>
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Calcitonin</t>
+          <t>Take a drug holiday, as for bisphosphonates</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>Alendronate</t>
+          <t>Switch to teriparatide for life</t>
         </is>
       </c>
       <c r="E37" s="16" t="inlineStr">
         <is>
-          <t>Teriparatide</t>
+          <t>Stop safely: its effect lasts years in bone</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>Raloxifene</t>
+          <t>Don’t just stop — transition to a bisphosphonate</t>
         </is>
       </c>
       <c r="G37" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I37" s="1" t="n"/>
@@ -3523,27 +3523,27 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>A patient on denosumab for 4 years wants to stop it because of the injections. What should the PA advise?</t>
+          <t>A patient with CrCl 25 mL/min has osteoporosis. Which drug class is contraindicated at this kidney function?</t>
         </is>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>
-          <t>Stop safely: its effect lasts years in bone</t>
+          <t>RANKL antibodies such as denosumab</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>Don’t just stop — transition to a bisphosphonate</t>
+          <t>PTH analogs such as teriparatide</t>
         </is>
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
-          <t>Switch to teriparatide for life</t>
+          <t>Bisphosphonates such as alendronate</t>
         </is>
       </c>
       <c r="F38" s="16" t="inlineStr">
         <is>
-          <t>Stop and start calcium only</t>
+          <t>Estrogen modulators such as raloxifene</t>
         </is>
       </c>
       <c r="G38" s="14" t="n">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="H38" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I38" s="1" t="n"/>
@@ -3580,35 +3580,35 @@
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>A patient with CrCl 25 mL/min has osteoporosis. Which drug class is contraindicated at this kidney function?</t>
+          <t>Why does raloxifene suit some patients with vertebral osteoporosis but not those whose main risk is hip fracture?</t>
         </is>
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>PTH analogs such as teriparatide</t>
+          <t>It reduces spine fractures but not hip fractures</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>Estrogen modulators such as raloxifene</t>
+          <t>It must be stopped after 2 years</t>
         </is>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
-          <t>Sclerostin antibodies such as romosozumab</t>
+          <t>It raises hip fracture risk through VTE</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>Bisphosphonates such as alendronate</t>
+          <t>It builds new bone only in the hip</t>
         </is>
       </c>
       <c r="G39" s="14" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I39" s="1" t="n"/>
@@ -3637,27 +3637,27 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>Why does raloxifene suit some patients with vertebral osteoporosis but not those whose main risk is hip fracture?</t>
+          <t>Raise uric acid: which is right?</t>
         </is>
       </c>
       <c r="C40" s="16" t="inlineStr">
         <is>
-          <t>It is contraindicated in all women over 65</t>
+          <t>Microtubules · best within 24 h · diarrhea · CYP3A4/P-gp</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>It raises hip fracture risk through VTE</t>
+          <t>RANKL antibody · stopping → rebound vertebral fractures</t>
         </is>
       </c>
       <c r="E40" s="16" t="inlineStr">
         <is>
-          <t>It reduces spine fractures but not hip fractures</t>
+          <t>Purine/fructose diet, beer, thiazide/loop diuretics, CKD</t>
         </is>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
-          <t>It must be stopped after 2 years</t>
+          <t>Hyperkalemia (burns, denervation, trauma); MH trigger</t>
         </is>
       </c>
       <c r="G40" s="14" t="n">
@@ -3694,31 +3694,31 @@
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>Raise uric acid: which is right?</t>
+          <t>Flare drugs: which is right?</t>
         </is>
       </c>
       <c r="C41" s="16" t="inlineStr">
         <is>
-          <t>Microtubules · best within 24 h · diarrhea · CYP3A4/P-gp</t>
+          <t>Formation vs. resorption (↑ RANKL)</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>RANKL antibody · stopping → rebound vertebral fractures</t>
+          <t>8 mg IV every 2 weeks; premedicate</t>
         </is>
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>Purine/fructose diet, beer, thiazide/loop diuretics, CKD</t>
+          <t>Colchicine, NSAIDs, corticosteroids</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>Hyperkalemia (burns, denervation, trauma); MH trigger</t>
+          <t>Colchicine or NSAID for 3–6 months</t>
         </is>
       </c>
       <c r="G41" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H41" s="18" t="inlineStr">
         <is>
@@ -3751,35 +3751,35 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>Flare drugs: which is right?</t>
+          <t>Urate-lowering drugs: which is right?</t>
         </is>
       </c>
       <c r="C42" s="16" t="inlineStr">
         <is>
-          <t>Formation vs. resorption (↑ RANKL)</t>
+          <t>CrCl &lt; 30–35 · ONJ, atypical femur fracture · holiday after 3–5 y</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>8 mg IV every 2 weeks; premedicate</t>
+          <t>Prednisone 30–50 mg/d × 1–2 days, taper 7–10 days; good in CKD</t>
         </is>
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
-          <t>Colchicine, NSAIDs, corticosteroids</t>
+          <t>Age, estrogen loss, glucocorticoids, low Ca/vitamin D, inactivity</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>Colchicine or NSAID for 3–6 months</t>
+          <t>Allopurinol, febuxostat (↓ production); probenecid (↑ excretion)</t>
         </is>
       </c>
       <c r="G42" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H42" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I42" s="1" t="n"/>
@@ -3808,27 +3808,27 @@
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>Urate-lowering drugs: which is right?</t>
+          <t>ULT in a flare?: which is right?</t>
         </is>
       </c>
       <c r="C43" s="16" t="inlineStr">
         <is>
-          <t>CrCl &lt; 30–35 · ONJ, atypical femur fracture · holiday after 3–5 y</t>
+          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Prednisone 30–50 mg/d × 1–2 days, taper 7–10 days; good in CKD</t>
+          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
         </is>
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
-          <t>Age, estrogen loss, glucocorticoids, low Ca/vitamin D, inactivity</t>
+          <t>RyR1 · malignant hyperthermia, NMS · hepatotoxic</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>Allopurinol, febuxostat (↓ production); probenecid (↑ excretion)</t>
+          <t>Never start or change — it can prolong the flare</t>
         </is>
       </c>
       <c r="G43" s="14" t="n">
@@ -3865,35 +3865,35 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>ULT in a flare?: which is right?</t>
+          <t>ULT prophylaxis: which is right?</t>
         </is>
       </c>
       <c r="C44" s="16" t="inlineStr">
         <is>
-          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
+          <t>Colchicine or NSAID for 3–6 months</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
+          <t>Formation vs. resorption (↑ RANKL)</t>
         </is>
       </c>
       <c r="E44" s="16" t="inlineStr">
         <is>
-          <t>RyR1 · malignant hyperthermia, NMS · hepatotoxic</t>
+          <t>8 mg IV every 2 weeks; premedicate</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>Never start or change — it can prolong the flare</t>
+          <t>Colchicine, NSAIDs, corticosteroids</t>
         </is>
       </c>
       <c r="G44" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H44" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I44" s="1" t="n"/>
@@ -3922,31 +3922,31 @@
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>ULT prophylaxis: which is right?</t>
+          <t>Colchicine: which is right?</t>
         </is>
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Colchicine or NSAID for 3–6 months</t>
+          <t>Microtubules · best within 24 h · diarrhea · CYP3A4/P-gp</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>Formation vs. resorption (↑ RANKL)</t>
+          <t>Purine/fructose diet, beer, thiazide/loop diuretics, CKD</t>
         </is>
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>8 mg IV every 2 weeks; premedicate</t>
+          <t>Hyperkalemia (burns, denervation, trauma); MH trigger</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>Colchicine, NSAIDs, corticosteroids</t>
+          <t>RANKL antibody · stopping → rebound vertebral fractures</t>
         </is>
       </c>
       <c r="G45" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H45" s="18" t="inlineStr">
         <is>
@@ -3979,35 +3979,35 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>Colchicine: which is right?</t>
+          <t>Febuxostat: which is right?</t>
         </is>
       </c>
       <c r="C46" s="16" t="inlineStr">
         <is>
-          <t>Microtubules · best within 24 h · diarrhea · CYP3A4/P-gp</t>
+          <t>20 mcg · 80 mcg SC daily; 2 years</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>Purine/fructose diet, beer, thiazide/loop diuretics, CKD</t>
+          <t>1.2 mg, then 0.6 mg 1 h later</t>
         </is>
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
-          <t>Hyperkalemia (burns, denervation, trauma); MH trigger</t>
+          <t>→ meprobamate · Schedule IV</t>
         </is>
       </c>
       <c r="F46" s="16" t="inlineStr">
         <is>
-          <t>RANKL antibody · stopping → rebound vertebral fractures</t>
+          <t>XO inhibitor · boxed CV death</t>
         </is>
       </c>
       <c r="G46" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H46" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I46" s="1" t="n"/>
@@ -4036,35 +4036,35 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>Febuxostat: which is right?</t>
+          <t>Probenecid: which is right?</t>
         </is>
       </c>
       <c r="C47" s="16" t="inlineStr">
         <is>
-          <t>20 mcg · 80 mcg SC daily; 2 years</t>
+          <t>600 IU/d adults; deficiency 1000–4000 IU/d or 50,000 IU/week</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>1.2 mg, then 0.6 mg 1 h later</t>
+          <t>Reverses rocuronium/vecuronium; backup contraception 7 days</t>
         </is>
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>→ meprobamate · Schedule IV</t>
+          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>XO inhibitor · boxed CV death</t>
+          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
         </is>
       </c>
       <c r="G47" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I47" s="1" t="n"/>
@@ -4093,27 +4093,27 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>Probenecid: which is right?</t>
+          <t>Pegloticase, rasburicase: which is right?</t>
         </is>
       </c>
       <c r="C48" s="16" t="inlineStr">
         <is>
-          <t>600 IU/d adults; deficiency 1000–4000 IU/d or 50,000 IU/week</t>
+          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>Reverses rocuronium/vecuronium; backup contraception 7 days</t>
+          <t>Full glass of water, fasting, upright 30 min</t>
         </is>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
+          <t>Uricase → allantoin · IV · no G6PD deficiency</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
+          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
         </is>
       </c>
       <c r="G48" s="14" t="n">
@@ -4150,12 +4150,12 @@
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>Pegloticase, rasburicase: which is right?</t>
+          <t>Spasticity vs. rigidity: which is right?</t>
         </is>
       </c>
       <c r="C49" s="16" t="inlineStr">
         <is>
-          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
+          <t>Spine, not hip; VTE; no hot-flush relief</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -4165,12 +4165,12 @@
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>Uricase → allantoin · IV · no G6PD deficiency</t>
+          <t>1 mg/kg IV, repeat; RyR1 (heart uses RyR2)</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
+          <t>Velocity-dependent (UMN) vs. constant tone</t>
         </is>
       </c>
       <c r="G49" s="14" t="n">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="H49" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I49" s="1" t="n"/>
@@ -4207,27 +4207,27 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>Spasticity vs. rigidity: which is right?</t>
+          <t>Peripheral relaxants: which is right?</t>
         </is>
       </c>
       <c r="C50" s="16" t="inlineStr">
         <is>
-          <t>Spine, not hip; VTE; no hot-flush relief</t>
+          <t>RyR1 · malignant hyperthermia, NMS · hepatotoxic</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>Full glass of water, fasting, upright 30 min</t>
+          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
         </is>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
-          <t>1 mg/kg IV, repeat; RyR1 (heart uses RyR2)</t>
+          <t>Never start or change — it can prolong the flare</t>
         </is>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
-          <t>Velocity-dependent (UMN) vs. constant tone</t>
+          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
         </is>
       </c>
       <c r="G50" s="14" t="n">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="H50" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I50" s="1" t="n"/>
@@ -4264,27 +4264,27 @@
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>Peripheral relaxants: which is right?</t>
+          <t>Tizanidine: which is right?</t>
         </is>
       </c>
       <c r="C51" s="16" t="inlineStr">
         <is>
-          <t>RyR1 · malignant hyperthermia, NMS · hepatotoxic</t>
+          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
+          <t>Prednisone 30–50 mg/d × 1–2 days, taper 7–10 days; good in CKD</t>
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>Never start or change — it can prolong the flare</t>
+          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
+          <t>600 IU/d adults; deficiency 1000–4000 IU/d or 50,000 IU/week</t>
         </is>
       </c>
       <c r="G51" s="14" t="n">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="H51" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I51" s="1" t="n"/>
@@ -4321,19 +4321,19 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>Tizanidine: which is right?</t>
+          <t>Cyclobenzaprine: which is right?</t>
         </is>
       </c>
       <c r="C52" s="16" t="inlineStr">
         <is>
+          <t>Prednisone 30–50 mg/d × 1–2 days, taper 7–10 days; good in CKD</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
           <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
         </is>
       </c>
-      <c r="D52" s="16" t="inlineStr">
-        <is>
-          <t>Prednisone 30–50 mg/d × 1–2 days, taper 7–10 days; good in CKD</t>
-        </is>
-      </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
           <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
-          <t>600 IU/d adults; deficiency 1000–4000 IU/d or 50,000 IU/week</t>
+          <t>Brainstem 5-HT2 · TCA-like anticholinergic · 2–3 weeks · Beers</t>
         </is>
       </c>
       <c r="G52" s="14" t="n">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="H52" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I52" s="1" t="n"/>
@@ -4378,35 +4378,35 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>Cyclobenzaprine: which is right?</t>
+          <t>Carisoprodol: which is right?</t>
         </is>
       </c>
       <c r="C53" s="16" t="inlineStr">
         <is>
-          <t>Prednisone 30–50 mg/d × 1–2 days, taper 7–10 days; good in CKD</t>
+          <t>→ meprobamate · Schedule IV</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
+          <t>XO inhibitor · boxed CV death</t>
         </is>
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
-          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
+          <t>20 mcg · 80 mcg SC daily; 2 years</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>Brainstem 5-HT2 · TCA-like anticholinergic · 2–3 weeks · Beers</t>
+          <t>1.2 mg, then 0.6 mg 1 h later</t>
         </is>
       </c>
       <c r="G53" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H53" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I53" s="1" t="n"/>
@@ -4435,35 +4435,35 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>Carisoprodol: which is right?</t>
+          <t>Dantrolene: which is right?</t>
         </is>
       </c>
       <c r="C54" s="16" t="inlineStr">
         <is>
-          <t>→ meprobamate · Schedule IV</t>
+          <t>Never start or change — it can prolong the flare</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>XO inhibitor · boxed CV death</t>
+          <t>RyR1 · malignant hyperthermia, NMS · hepatotoxic</t>
         </is>
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
-          <t>20 mcg · 80 mcg SC daily; 2 years</t>
+          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
         </is>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
-          <t>1.2 mg, then 0.6 mg 1 h later</t>
+          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
         </is>
       </c>
       <c r="G54" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H54" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I54" s="1" t="n"/>
@@ -4492,35 +4492,35 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>Dantrolene: which is right?</t>
+          <t>Malignant hyperthermia triggers: which is right?</t>
         </is>
       </c>
       <c r="C55" s="16" t="inlineStr">
         <is>
-          <t>Never start or change — it can prolong the flare</t>
+          <t>Volatile anesthetics, succinylcholine</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>RyR1 · malignant hyperthermia, NMS · hepatotoxic</t>
+          <t>PTH 1-34 · anabolic · 2 years lifetime</t>
         </is>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
-          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
+          <t>Colchicine, NSAIDs, corticosteroids</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
-          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
+          <t>8 mg IV every 2 weeks; premedicate</t>
         </is>
       </c>
       <c r="G55" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H55" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I55" s="1" t="n"/>
@@ -4549,31 +4549,31 @@
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>Malignant hyperthermia triggers: which is right?</t>
+          <t>Osteoporosis risk: which is right?</t>
         </is>
       </c>
       <c r="C56" s="16" t="inlineStr">
         <is>
-          <t>Volatile anesthetics, succinylcholine</t>
+          <t>Age, estrogen loss, glucocorticoids, low Ca/vitamin D, inactivity</t>
         </is>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>PTH 1-34 · anabolic · 2 years lifetime</t>
+          <t>CrCl &lt; 30–35 · ONJ, atypical femur fracture · holiday after 3–5 y</t>
         </is>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
-          <t>Colchicine, NSAIDs, corticosteroids</t>
+          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
         </is>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
-          <t>8 mg IV every 2 weeks; premedicate</t>
+          <t>Allopurinol, febuxostat (↓ production); probenecid (↑ excretion)</t>
         </is>
       </c>
       <c r="G56" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H56" s="18" t="inlineStr">
         <is>
@@ -4606,27 +4606,27 @@
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>Osteoporosis risk: which is right?</t>
+          <t>PTH loop: which is right?</t>
         </is>
       </c>
       <c r="C57" s="16" t="inlineStr">
         <is>
-          <t>Age, estrogen loss, glucocorticoids, low Ca/vitamin D, inactivity</t>
+          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>CrCl &lt; 30–35 · ONJ, atypical femur fracture · holiday after 3–5 y</t>
+          <t>Sclerostin antibody · builds + limits resorption · boxed MI/stroke/CV death</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
-          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
+          <t>Start 2–3 weeks after an attack; urine pH &gt; 6.0; ↓ penicillin secretion</t>
         </is>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>Allopurinol, febuxostat (↓ production); probenecid (↑ excretion)</t>
+          <t>↓ Ca → PTH → bone resorption, renal reabsorption, vitamin D gut absorption</t>
         </is>
       </c>
       <c r="G57" s="14" t="n">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="H57" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I57" s="1" t="n"/>
@@ -4663,31 +4663,31 @@
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>PTH loop: which is right?</t>
+          <t>Intermittent vs. continuous PTH: which is right?</t>
         </is>
       </c>
       <c r="C58" s="16" t="inlineStr">
         <is>
-          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
+          <t>8 mg IV every 2 weeks; premedicate</t>
         </is>
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>Sclerostin antibody · builds + limits resorption · boxed MI/stroke/CV death</t>
+          <t>Colchicine, NSAIDs, corticosteroids</t>
         </is>
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
-          <t>Start 2–3 weeks after an attack; urine pH &gt; 6.0; ↓ penicillin secretion</t>
+          <t>Colchicine or NSAID for 3–6 months</t>
         </is>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
-          <t>↓ Ca → PTH → bone resorption, renal reabsorption, vitamin D gut absorption</t>
+          <t>Formation vs. resorption (↑ RANKL)</t>
         </is>
       </c>
       <c r="G58" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H58" s="18" t="inlineStr">
         <is>
@@ -4720,35 +4720,35 @@
       </c>
       <c r="B59" s="16" t="inlineStr">
         <is>
-          <t>Intermittent vs. continuous PTH: which is right?</t>
+          <t>Bisphosphonate counseling: which is right?</t>
         </is>
       </c>
       <c r="C59" s="16" t="inlineStr">
         <is>
-          <t>8 mg IV every 2 weeks; premedicate</t>
+          <t>Velocity-dependent (UMN) vs. constant tone</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>Colchicine, NSAIDs, corticosteroids</t>
+          <t>Uricase → allantoin · IV · no G6PD deficiency</t>
         </is>
       </c>
       <c r="E59" s="16" t="inlineStr">
         <is>
-          <t>Colchicine or NSAID for 3–6 months</t>
+          <t>Full glass of water, fasting, upright 30 min</t>
         </is>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>Formation vs. resorption (↑ RANKL)</t>
+          <t>1 mg/kg IV, repeat; RyR1 (heart uses RyR2)</t>
         </is>
       </c>
       <c r="G59" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H59" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I59" s="1" t="n"/>
@@ -4777,27 +4777,27 @@
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>Bisphosphonate counseling: which is right?</t>
+          <t>Bisphosphonate limits: which is right?</t>
         </is>
       </c>
       <c r="C60" s="16" t="inlineStr">
         <is>
-          <t>Velocity-dependent (UMN) vs. constant tone</t>
+          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>Uricase → allantoin · IV · no G6PD deficiency</t>
+          <t>Age, estrogen loss, glucocorticoids, low Ca/vitamin D, inactivity</t>
         </is>
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
-          <t>Full glass of water, fasting, upright 30 min</t>
+          <t>CrCl &lt; 30–35 · ONJ, atypical femur fracture · holiday after 3–5 y</t>
         </is>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
-          <t>1 mg/kg IV, repeat; RyR1 (heart uses RyR2)</t>
+          <t>Allopurinol, febuxostat (↓ production); probenecid (↑ excretion)</t>
         </is>
       </c>
       <c r="G60" s="14" t="n">
@@ -4834,27 +4834,27 @@
       </c>
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>Bisphosphonate limits: which is right?</t>
+          <t>Denosumab: which is right?</t>
         </is>
       </c>
       <c r="C61" s="16" t="inlineStr">
         <is>
-          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
+          <t>Hyperkalemia (burns, denervation, trauma); MH trigger</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Age, estrogen loss, glucocorticoids, low Ca/vitamin D, inactivity</t>
+          <t>Microtubules · best within 24 h · diarrhea · CYP3A4/P-gp</t>
         </is>
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
-          <t>CrCl &lt; 30–35 · ONJ, atypical femur fracture · holiday after 3–5 y</t>
+          <t>RANKL antibody · stopping → rebound vertebral fractures</t>
         </is>
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
-          <t>Allopurinol, febuxostat (↓ production); probenecid (↑ excretion)</t>
+          <t>Purine/fructose diet, beer, thiazide/loop diuretics, CKD</t>
         </is>
       </c>
       <c r="G61" s="14" t="n">
@@ -4891,35 +4891,35 @@
       </c>
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>Denosumab: which is right?</t>
+          <t>Teriparatide: which is right?</t>
         </is>
       </c>
       <c r="C62" s="16" t="inlineStr">
         <is>
-          <t>Hyperkalemia (burns, denervation, trauma); MH trigger</t>
+          <t>Spine, not hip; VTE; no hot-flush relief</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>Microtubules · best within 24 h · diarrhea · CYP3A4/P-gp</t>
+          <t>Colchicine, NSAIDs, corticosteroids</t>
         </is>
       </c>
       <c r="E62" s="16" t="inlineStr">
         <is>
-          <t>RANKL antibody · stopping → rebound vertebral fractures</t>
+          <t>Volatile anesthetics, succinylcholine</t>
         </is>
       </c>
       <c r="F62" s="16" t="inlineStr">
         <is>
-          <t>Purine/fructose diet, beer, thiazide/loop diuretics, CKD</t>
+          <t>PTH 1-34 · anabolic · 2 years lifetime</t>
         </is>
       </c>
       <c r="G62" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H62" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I62" s="1" t="n"/>
@@ -4948,35 +4948,35 @@
       </c>
       <c r="B63" s="16" t="inlineStr">
         <is>
-          <t>Teriparatide: which is right?</t>
+          <t>Romosozumab: which is right?</t>
         </is>
       </c>
       <c r="C63" s="16" t="inlineStr">
         <is>
-          <t>Spine, not hip; VTE; no hot-flush relief</t>
+          <t>Start 2–3 weeks after an attack; urine pH &gt; 6.0; ↓ penicillin secretion</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>Colchicine, NSAIDs, corticosteroids</t>
+          <t>↓ Ca → PTH → bone resorption, renal reabsorption, vitamin D gut absorption</t>
         </is>
       </c>
       <c r="E63" s="16" t="inlineStr">
         <is>
-          <t>Volatile anesthetics, succinylcholine</t>
+          <t>Sclerostin antibody · builds + limits resorption · boxed MI/stroke/CV death</t>
         </is>
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
-          <t>PTH 1-34 · anabolic · 2 years lifetime</t>
+          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
         </is>
       </c>
       <c r="G63" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H63" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I63" s="1" t="n"/>
@@ -5005,27 +5005,27 @@
       </c>
       <c r="B64" s="16" t="inlineStr">
         <is>
-          <t>Romosozumab: which is right?</t>
+          <t>Raloxifene: which is right?</t>
         </is>
       </c>
       <c r="C64" s="16" t="inlineStr">
         <is>
-          <t>Start 2–3 weeks after an attack; urine pH &gt; 6.0; ↓ penicillin secretion</t>
+          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
         </is>
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>↓ Ca → PTH → bone resorption, renal reabsorption, vitamin D gut absorption</t>
+          <t>Full glass of water, fasting, upright 30 min</t>
         </is>
       </c>
       <c r="E64" s="16" t="inlineStr">
         <is>
-          <t>Sclerostin antibody · builds + limits resorption · boxed MI/stroke/CV death</t>
+          <t>Uricase → allantoin · IV · no G6PD deficiency</t>
         </is>
       </c>
       <c r="F64" s="16" t="inlineStr">
         <is>
-          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
+          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
         </is>
       </c>
       <c r="G64" s="14" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="H64" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I64" s="1" t="n"/>
@@ -5062,27 +5062,27 @@
       </c>
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>Raloxifene: which is right?</t>
+          <t>Allopurinol dosing: which is right?</t>
         </is>
       </c>
       <c r="C65" s="16" t="inlineStr">
         <is>
-          <t>SERM · VTE, hot flashes · ↓ breast cancer risk</t>
+          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>Full glass of water, fasting, upright 30 min</t>
+          <t>Allopurinol, febuxostat (↓ production); probenecid (↑ excretion)</t>
         </is>
       </c>
       <c r="E65" s="16" t="inlineStr">
         <is>
-          <t>Uricase → allantoin · IV · no G6PD deficiency</t>
+          <t>CrCl &lt; 30–35 · ONJ, atypical femur fracture · holiday after 3–5 y</t>
         </is>
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>Dantrolene (muscle), botulinum toxin (junction)</t>
+          <t>Age, estrogen loss, glucocorticoids, low Ca/vitamin D, inactivity</t>
         </is>
       </c>
       <c r="G65" s="14" t="n">
@@ -5119,35 +5119,35 @@
       </c>
       <c r="B66" s="16" t="inlineStr">
         <is>
-          <t>Allopurinol dosing: which is right?</t>
+          <t>Colchicine flare dose: which is right?</t>
         </is>
       </c>
       <c r="C66" s="16" t="inlineStr">
         <is>
-          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
+          <t>XO inhibitor · boxed CV death</t>
         </is>
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>Allopurinol, febuxostat (↓ production); probenecid (↑ excretion)</t>
+          <t>→ meprobamate · Schedule IV</t>
         </is>
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
-          <t>CrCl &lt; 30–35 · ONJ, atypical femur fracture · holiday after 3–5 y</t>
+          <t>20 mcg · 80 mcg SC daily; 2 years</t>
         </is>
       </c>
       <c r="F66" s="16" t="inlineStr">
         <is>
-          <t>Age, estrogen loss, glucocorticoids, low Ca/vitamin D, inactivity</t>
+          <t>1.2 mg, then 0.6 mg 1 h later</t>
         </is>
       </c>
       <c r="G66" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H66" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I66" s="1" t="n"/>
@@ -5176,35 +5176,35 @@
       </c>
       <c r="B67" s="16" t="inlineStr">
         <is>
-          <t>Colchicine flare dose: which is right?</t>
+          <t>Gout steroid option: which is right?</t>
         </is>
       </c>
       <c r="C67" s="16" t="inlineStr">
         <is>
-          <t>XO inhibitor · boxed CV death</t>
+          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>→ meprobamate · Schedule IV</t>
+          <t>Prednisone 30–50 mg/d × 1–2 days, taper 7–10 days; good in CKD</t>
         </is>
       </c>
       <c r="E67" s="16" t="inlineStr">
         <is>
-          <t>20 mcg · 80 mcg SC daily; 2 years</t>
+          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
         </is>
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
-          <t>1.2 mg, then 0.6 mg 1 h later</t>
+          <t>Brainstem 5-HT2 · TCA-like anticholinergic · 2–3 weeks · Beers</t>
         </is>
       </c>
       <c r="G67" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H67" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I67" s="1" t="n"/>
@@ -5233,35 +5233,35 @@
       </c>
       <c r="B68" s="16" t="inlineStr">
         <is>
-          <t>Gout steroid option: which is right?</t>
+          <t>Pegloticase dose: which is right?</t>
         </is>
       </c>
       <c r="C68" s="16" t="inlineStr">
         <is>
-          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
+          <t>Colchicine, NSAIDs, corticosteroids</t>
         </is>
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>Prednisone 30–50 mg/d × 1–2 days, taper 7–10 days; good in CKD</t>
+          <t>Colchicine or NSAID for 3–6 months</t>
         </is>
       </c>
       <c r="E68" s="16" t="inlineStr">
         <is>
-          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
+          <t>Formation vs. resorption (↑ RANKL)</t>
         </is>
       </c>
       <c r="F68" s="16" t="inlineStr">
         <is>
-          <t>Brainstem 5-HT2 · TCA-like anticholinergic · 2–3 weeks · Beers</t>
+          <t>8 mg IV every 2 weeks; premedicate</t>
         </is>
       </c>
       <c r="G68" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H68" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I68" s="1" t="n"/>
@@ -5290,35 +5290,35 @@
       </c>
       <c r="B69" s="16" t="inlineStr">
         <is>
-          <t>Pegloticase dose: which is right?</t>
+          <t>Probenecid: which is right?</t>
         </is>
       </c>
       <c r="C69" s="16" t="inlineStr">
         <is>
-          <t>Colchicine, NSAIDs, corticosteroids</t>
+          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>Colchicine or NSAID for 3–6 months</t>
+          <t>Start 2–3 weeks after an attack; urine pH &gt; 6.0; ↓ penicillin secretion</t>
         </is>
       </c>
       <c r="E69" s="16" t="inlineStr">
         <is>
-          <t>Formation vs. resorption (↑ RANKL)</t>
+          <t>↓ Ca → PTH → bone resorption, renal reabsorption, vitamin D gut absorption</t>
         </is>
       </c>
       <c r="F69" s="16" t="inlineStr">
         <is>
-          <t>8 mg IV every 2 weeks; premedicate</t>
+          <t>Sclerostin antibody · builds + limits resorption · boxed MI/stroke/CV death</t>
         </is>
       </c>
       <c r="G69" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H69" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I69" s="1" t="n"/>
@@ -5347,27 +5347,27 @@
       </c>
       <c r="B70" s="16" t="inlineStr">
         <is>
-          <t>Probenecid: which is right?</t>
+          <t>Dantrolene in MH: which is right?</t>
         </is>
       </c>
       <c r="C70" s="16" t="inlineStr">
         <is>
-          <t>Start 100 mg/d (≤50 in CKD); titrate to uric acid &lt;6 mg/dL; max 800</t>
+          <t>Spine, not hip; VTE; no hot-flush relief</t>
         </is>
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>Start 2–3 weeks after an attack; urine pH &gt; 6.0; ↓ penicillin secretion</t>
+          <t>1 mg/kg IV, repeat; RyR1 (heart uses RyR2)</t>
         </is>
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
-          <t>↓ Ca → PTH → bone resorption, renal reabsorption, vitamin D gut absorption</t>
+          <t>Full glass of water, fasting, upright 30 min</t>
         </is>
       </c>
       <c r="F70" s="16" t="inlineStr">
         <is>
-          <t>Sclerostin antibody · builds + limits resorption · boxed MI/stroke/CV death</t>
+          <t>Velocity-dependent (UMN) vs. constant tone</t>
         </is>
       </c>
       <c r="G70" s="14" t="n">
@@ -5404,27 +5404,27 @@
       </c>
       <c r="B71" s="16" t="inlineStr">
         <is>
-          <t>Dantrolene in MH: which is right?</t>
+          <t>Succinylcholine dangers: which is right?</t>
         </is>
       </c>
       <c r="C71" s="16" t="inlineStr">
         <is>
-          <t>Spine, not hip; VTE; no hot-flush relief</t>
+          <t>Purine/fructose diet, beer, thiazide/loop diuretics, CKD</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>1 mg/kg IV, repeat; RyR1 (heart uses RyR2)</t>
+          <t>Hyperkalemia (burns, denervation, trauma); MH trigger</t>
         </is>
       </c>
       <c r="E71" s="16" t="inlineStr">
         <is>
-          <t>Full glass of water, fasting, upright 30 min</t>
+          <t>Microtubules · best within 24 h · diarrhea · CYP3A4/P-gp</t>
         </is>
       </c>
       <c r="F71" s="16" t="inlineStr">
         <is>
-          <t>Velocity-dependent (UMN) vs. constant tone</t>
+          <t>RANKL antibody · stopping → rebound vertebral fractures</t>
         </is>
       </c>
       <c r="G71" s="14" t="n">
@@ -5461,27 +5461,27 @@
       </c>
       <c r="B72" s="16" t="inlineStr">
         <is>
-          <t>Succinylcholine dangers: which is right?</t>
+          <t>Sugammadex: which is right?</t>
         </is>
       </c>
       <c r="C72" s="16" t="inlineStr">
         <is>
-          <t>Purine/fructose diet, beer, thiazide/loop diuretics, CKD</t>
+          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
         </is>
       </c>
       <c r="D72" s="16" t="inlineStr">
         <is>
-          <t>Hyperkalemia (burns, denervation, trauma); MH trigger</t>
+          <t>Reverses rocuronium/vecuronium; backup contraception 7 days</t>
         </is>
       </c>
       <c r="E72" s="16" t="inlineStr">
         <is>
-          <t>Microtubules · best within 24 h · diarrhea · CYP3A4/P-gp</t>
+          <t>600 IU/d adults; deficiency 1000–4000 IU/d or 50,000 IU/week</t>
         </is>
       </c>
       <c r="F72" s="16" t="inlineStr">
         <is>
-          <t>RANKL antibody · stopping → rebound vertebral fractures</t>
+          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
         </is>
       </c>
       <c r="G72" s="14" t="n">
@@ -5518,35 +5518,35 @@
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>Sugammadex: which is right?</t>
+          <t>Teriparatide · abaloparatide: which is right?</t>
         </is>
       </c>
       <c r="C73" s="16" t="inlineStr">
         <is>
-          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
+          <t>Formation vs. resorption (↑ RANKL)</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Reverses rocuronium/vecuronium; backup contraception 7 days</t>
+          <t>Colchicine or NSAID for 3–6 months</t>
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
-          <t>600 IU/d adults; deficiency 1000–4000 IU/d or 50,000 IU/week</t>
+          <t>8 mg IV every 2 weeks; premedicate</t>
         </is>
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
-          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
+          <t>20 mcg · 80 mcg SC daily; 2 years</t>
         </is>
       </c>
       <c r="G73" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H73" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I73" s="1" t="n"/>
@@ -5575,35 +5575,35 @@
       </c>
       <c r="B74" s="16" t="inlineStr">
         <is>
-          <t>Teriparatide · abaloparatide: which is right?</t>
+          <t>Raloxifene: which is right?</t>
         </is>
       </c>
       <c r="C74" s="16" t="inlineStr">
         <is>
-          <t>Formation vs. resorption (↑ RANKL)</t>
+          <t>Spine, not hip; VTE; no hot-flush relief</t>
         </is>
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>Colchicine or NSAID for 3–6 months</t>
+          <t>Velocity-dependent (UMN) vs. constant tone</t>
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr">
         <is>
-          <t>8 mg IV every 2 weeks; premedicate</t>
+          <t>1 mg/kg IV, repeat; RyR1 (heart uses RyR2)</t>
         </is>
       </c>
       <c r="F74" s="16" t="inlineStr">
         <is>
-          <t>20 mcg · 80 mcg SC daily; 2 years</t>
+          <t>PTH 1-34 · anabolic · 2 years lifetime</t>
         </is>
       </c>
       <c r="G74" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H74" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I74" s="1" t="n"/>
@@ -5632,27 +5632,27 @@
       </c>
       <c r="B75" s="16" t="inlineStr">
         <is>
-          <t>Raloxifene: which is right?</t>
+          <t>Vitamin D: which is right?</t>
         </is>
       </c>
       <c r="C75" s="16" t="inlineStr">
         <is>
-          <t>Spine, not hip; VTE; no hot-flush relief</t>
+          <t>600 IU/d adults; deficiency 1000–4000 IU/d or 50,000 IU/week</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Velocity-dependent (UMN) vs. constant tone</t>
+          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
         <is>
-          <t>1 mg/kg IV, repeat; RyR1 (heart uses RyR2)</t>
+          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
         </is>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>PTH 1-34 · anabolic · 2 years lifetime</t>
+          <t>Reverses rocuronium/vecuronium; backup contraception 7 days</t>
         </is>
       </c>
       <c r="G75" s="14" t="n">
@@ -5684,42 +5684,14 @@
       <c r="AA75" s="1" t="n"/>
     </row>
     <row r="76" ht="25.5" customHeight="1">
-      <c r="A76" s="11" t="n">
-        <v>68</v>
-      </c>
-      <c r="B76" s="16" t="inlineStr">
-        <is>
-          <t>Vitamin D: which is right?</t>
-        </is>
-      </c>
-      <c r="C76" s="16" t="inlineStr">
-        <is>
-          <t>600 IU/d adults; deficiency 1000–4000 IU/d or 50,000 IU/week</t>
-        </is>
-      </c>
-      <c r="D76" s="16" t="inlineStr">
-        <is>
-          <t>α2 agonist · hypotension, LFTs · no ciprofloxacin/fluvoxamine</t>
-        </is>
-      </c>
-      <c r="E76" s="16" t="inlineStr">
-        <is>
-          <t>URAT1 block · hydrate · no uric acid stones/renal impairment</t>
-        </is>
-      </c>
-      <c r="F76" s="16" t="inlineStr">
-        <is>
-          <t>Reverses rocuronium/vecuronium; backup contraception 7 days</t>
-        </is>
-      </c>
-      <c r="G76" s="14" t="n">
-        <v>30</v>
-      </c>
-      <c r="H76" s="18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="A76" s="11" t="n"/>
+      <c r="B76" s="16" t="n"/>
+      <c r="C76" s="16" t="n"/>
+      <c r="D76" s="16" t="n"/>
+      <c r="E76" s="16" t="n"/>
+      <c r="F76" s="16" t="n"/>
+      <c r="G76" s="14" t="n"/>
+      <c r="H76" s="18" t="n"/>
       <c r="I76" s="1" t="n"/>
       <c r="J76" s="1" t="n"/>
       <c r="K76" s="1" t="n"/>

</xml_diff>